<commit_message>
[v1] Wolves in the Chetwood: validated and locked (drain=18, spike=75, spikeiv=9, boss=60000)
Validated at party Lv3, 5000 runs: Lv3 food 6%, Lv4 81%, Lv6 91%, Lv7 98%, Lv8 ~100%.
Needs max Hearthkeeper food (Lv4) for a real chance. Encounter Builder updated to match.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sim/HearthCraft_Encounter_Builder.xlsx
+++ b/tools/sim/HearthCraft_Encounter_Builder.xlsx
@@ -1317,12 +1317,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF4A2F1A"/>
   </sheetPr>
   <dimension ref="A1:Q18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -1339,22 +1339,22 @@
     <col min="17" max="17" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ns3:dyDescent="0.25">
       <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" ns3:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" ns3:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ns3:dyDescent="0.25">
       <c r="A5" s="18" t="s">
         <v>3</v>
       </c>
@@ -1407,7 +1407,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" ns3:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>20</v>
       </c>
@@ -1460,7 +1460,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" ns3:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>24</v>
       </c>
@@ -1477,16 +1477,16 @@
         <v>1500</v>
       </c>
       <c r="F7" s="19">
-        <v>55000</v>
+        <v>60000</v>
       </c>
       <c r="G7" s="19">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H7" s="19">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="I7" s="19">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J7" s="19">
         <v>0</v>
@@ -1513,7 +1513,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" ns3:dyDescent="0.25">
       <c r="A8" s="20" t="s">
         <v>26</v>
       </c>
@@ -1566,7 +1566,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" ns3:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>29</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" ns3:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>31</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" ns3:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>33</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ns3:dyDescent="0.25">
       <c r="A12" s="20" t="s">
         <v>35</v>
       </c>
@@ -1778,7 +1778,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" ns3:dyDescent="0.25">
       <c r="A13" s="20" t="s">
         <v>38</v>
       </c>
@@ -1831,7 +1831,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" ns3:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>40</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" ns3:dyDescent="0.25">
       <c r="A15" s="20" t="s">
         <v>42</v>
       </c>
@@ -1937,7 +1937,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" ns3:dyDescent="0.25">
       <c r="A16" s="20" t="s">
         <v>44</v>
       </c>
@@ -1990,7 +1990,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" ns3:dyDescent="0.25">
       <c r="A17" s="20" t="s">
         <v>46</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" ns3:dyDescent="0.25">
       <c r="A18" s="20" t="s">
         <v>48</v>
       </c>

</xml_diff>

<commit_message>
[v1] Encounter Builder: add winCurve + simCmd columns for validated encounters
R = win rate ladder by food level, S = exact sim command to reproduce.
Neekerbreekers and Wolves populated; placeholders left blank.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/sim/HearthCraft_Encounter_Builder.xlsx
+++ b/tools/sim/HearthCraft_Encounter_Builder.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="268">
   <si>
     <t>SIM TUNING SHEET — one row per encounter · columns map 1:1 to simulator controls</t>
   </si>
@@ -837,6 +837,24 @@
   </si>
   <si>
     <t>A cry in the dark, and a deathly cold. It cannot be slain — hold, keep the light, and endure until it withdraws.</t>
+  </si>
+  <si>
+    <t>winCurve</t>
+  </si>
+  <si>
+    <t>simCmd</t>
+  </si>
+  <si>
+    <t>Lv1=25%  Lv2=66%  Lv3=98%  Lv4=100%</t>
+  </si>
+  <si>
+    <t>node run_sim.js --runs 5000 --level 3 --duration 1500 --boss 50000 --drain 12 --spike 75 --spikeiv 13 --rlevel N</t>
+  </si>
+  <si>
+    <t>Lv3=6%  Lv4=81%  Lv6=91%  Lv7=98%  Lv8=100%</t>
+  </si>
+  <si>
+    <t>node run_sim.js --runs 5000 --level 3 --duration 1500 --boss 60000 --drain 18 --spike 75 --spikeiv 9 --rlevel N</t>
   </si>
 </sst>
 </file>
@@ -1406,6 +1424,12 @@
       <c r="Q5" s="18" t="s">
         <v>19</v>
       </c>
+      <c r="R5" t="s">
+        <v>262</v>
+      </c>
+      <c r="S5" t="s">
+        <v>263</v>
+      </c>
     </row>
     <row r="6" spans="1:17" ns3:dyDescent="0.25">
       <c r="A6" s="19" t="s">
@@ -1459,6 +1483,12 @@
       <c r="Q6" s="19" t="s">
         <v>23</v>
       </c>
+      <c r="R6" t="s">
+        <v>264</v>
+      </c>
+      <c r="S6" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="7" spans="1:17" ns3:dyDescent="0.25">
       <c r="A7" s="19" t="s">
@@ -1511,6 +1541,12 @@
       </c>
       <c r="Q7" s="19" t="s">
         <v>23</v>
+      </c>
+      <c r="R7" t="s">
+        <v>266</v>
+      </c>
+      <c r="S7" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="8" spans="1:17" ns3:dyDescent="0.25">

</xml_diff>